<commit_message>
Enrichit les 97 lieux : horaires, contact, site web, note/avis
Recherche web sur les infos absentes de benin_contenu_curation.xlsx
(horaires, téléphone, site web, note Google/TripAdvisor). Corrige au
passage plusieurs erreurs trouvées : localisation de la Forêt classée
de la Lama (Atlantique/Zou, pas Ouémé) et de Wari-Maro (Borgou/Donga,
pas Collines), renommage Basilique -> Église Sainte Rita, fusion des
doublons Fête de la Gani/Gaani et Palais/Musée d'Abomey, suppression
de l'Hôtel Arnogos (localisation introuvable en ligne).

Ajoute website/rating/reviews_count au modèle Lieu et à la fiche
détaillée ; horaires passe de jsonb (jamais peuplé) à text.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benin_contenu_curation.xlsx
+++ b/benin_contenu_curation.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:O43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -549,6 +549,36 @@
           <t>Statut</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Horaires</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Téléphone</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Site web</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Nb avis</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Remarque</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -561,7 +591,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Basilique Sainte Rita</t>
+          <t>Église Sainte Rita</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -639,6 +669,27 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Musée principal (Zongo/Haie Vive) : lun 14h-19h, mar-sam 10h-19h, fermé dim. LAB (Fidjrossè) : lun-ven ~9h-18h, fermé dim.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>+229 91 20 70 19</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.fondation-zinsou.org</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="N3" t="n">
+        <v>88</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -684,6 +735,12 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="M4" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="N4" t="n">
+        <v>72</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -729,6 +786,12 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="M5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N5" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -774,6 +837,17 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>+229 21 38 17 84</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="N6" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -819,6 +893,17 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>9h-18h tous les jours</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="N7" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -864,6 +949,22 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Tous les jours, environ 8h-19h</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>+229 41 44 87 06</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="N8" t="n">
+        <v>142</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -909,6 +1010,12 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="M9" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="N9" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -954,6 +1061,22 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>+229 21 34 10 21</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>4</v>
+      </c>
+      <c r="N10" t="n">
+        <v>79</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Possiblement fermé pour rénovation depuis 2026 — vérifier avant de s'y rendre.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -999,6 +1122,12 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="M11" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="N11" t="n">
+        <v>69</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1044,6 +1173,12 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="M12" t="n">
+        <v>4</v>
+      </c>
+      <c r="N12" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1089,6 +1224,17 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>+229 96 53 60 42</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="N13" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1134,6 +1280,17 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>+229 20 21 25 54</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="N14" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1179,6 +1336,21 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Visites guidées lun-ven 8h30/10h30/15h30/17h, sam 8h30/10h30/16h</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>+229 01 60 93 33 34</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://songhai.org</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1224,6 +1396,11 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Messes semaine 6h, 12h45, 18h ; dimanche 7h, 9h, 10h30, 19h</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1314,6 +1491,11 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>En travaux de réhabilitation — accessibilité à vérifier.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1359,6 +1541,11 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Patrimoine culturel immatériel (UNESCO) ; le berceau historique documenté est plutôt Kétou/Savè.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1449,6 +1636,22 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Tous les jours, 9h-18h</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>+229 22 50 03 14</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="N21" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1457,21 +1660,21 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Musée historique d'Abomey</t>
+          <t>Place Béhanzin (Place Goho)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Site touristique</t>
+          <t>Loisir</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Musée dans l'ancien palais royal, artefacts et trônes royaux.</t>
+          <t>Place centrale avec statue du roi Béhanzin, symbole de résistance.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1481,32 +1684,43 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>7.1863091, 1.9943789</t>
+          <t>7.1842529, 2.0078158</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1863091,1.9943789</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1842529,2.0078158</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="M22" t="n">
+        <v>4</v>
+      </c>
+      <c r="N22" t="n">
+        <v>5</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Un état d'entretien dégradé a été signalé par la presse locale.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Zou</t>
+          <t>Atlantique/Zou</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Place Béhanzin (Place Goho)</t>
+          <t>Forêt classée de la Lama</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1516,22 +1730,22 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Place centrale avec statue du roi Béhanzin, symbole de résistance.</t>
+          <t>Grande forêt naturelle, observation d'animaux et de flore variée.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Abomey, Zou</t>
+          <t>Toffo, Atlantique / Zogbodomey, Zou</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>7.1842529, 2.0078158</t>
+          <t>6.9179281, 2.1662158</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1842529,2.0078158</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.9179281,2.1662158</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1543,45 +1757,50 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Zou</t>
+          <t>Collines</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Forêt classée de la Lama</t>
+          <t>Grotte mariale de Dassa-Zoumé</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Loisir</t>
+          <t>Site touristique</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Grande forêt naturelle, observation d'animaux et de flore variée.</t>
+          <t>Lieu de pèlerinage catholique niché dans les collines.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Zou/Ouémé (zone Lama)</t>
+          <t>Dassa-Zoumé, Collines</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>6.9179281, 2.1662158</t>
+          <t>7.7752876, 2.1865136</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.9179281,2.1662158</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.7752876,2.1865136</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Ouvert toute l'année ; grand pèlerinage fin août</t>
         </is>
       </c>
     </row>
@@ -1592,11 +1811,11 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Grotte mariale de Dassa-Zoumé</t>
+          <t>Savalou (ville historique, culte vaudou)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1606,22 +1825,22 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Lieu de pèlerinage catholique niché dans les collines.</t>
+          <t>Ville traditionnelle marquée par la royauté locale et le culte vaudou.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Dassa-Zoumé, Collines</t>
+          <t>Savalou, Collines</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>7.7752876, 2.1865136</t>
+          <t>7.9301365, 1.9710284</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.7752876,2.1865136</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.9301365,1.9710284</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1633,40 +1852,40 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Collines</t>
+          <t>Mono</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Savalou (ville historique, culte vaudou)</t>
+          <t>Plage de Grand-Popo</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Site touristique</t>
+          <t>Loisir</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Ville traditionnelle marquée par la royauté locale et le culte vaudou.</t>
+          <t>Plage réputée du littoral béninois, tourisme balnéaire.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Savalou, Collines</t>
+          <t>Grand-Popo, Mono</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>7.9301365, 1.9710284</t>
+          <t>6.2639324, 1.7417143</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.9301365,1.9710284</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2639324,1.7417143</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1682,41 +1901,51 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Plage de Grand-Popo</t>
+          <t>Village de Possotomè</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Loisir</t>
+          <t>Site touristique</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Plage réputée du littoral béninois, tourisme balnéaire.</t>
+          <t>Village au bord du lac Ahémé, source d'eau thermale.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Grand-Popo, Mono</t>
+          <t>Possotomè, Bopa, Mono</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>6.2639324, 1.7417143</t>
+          <t>6.520838, 1.9625132</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2639324,1.7417143</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.520838,1.9625132</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>+229 95 28 52 20</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://www.ecobenin.org/possotome</t>
         </is>
       </c>
     </row>
@@ -1727,11 +1956,11 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Village de Possotomè</t>
+          <t>Bouche du Roy</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1741,28 +1970,44 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Village au bord du lac Ahémé, source d'eau thermale.</t>
+          <t>Embouchure spectaculaire entre océan, lagune et mangrove.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Possotomè, Bopa, Mono</t>
+          <t>Grand-Popo, Mono</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>6.520838, 1.9625132</t>
+          <t>6.2922216, 1.917286</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.520838,1.9625132</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2922216,1.917286</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>+229 60 63 08 18</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://www.boucheduroy.bj</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>4</v>
+      </c>
+      <c r="N28" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -1772,11 +2017,11 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Bouche du Roy</t>
+          <t>Ville de Lokossa</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1786,42 +2031,47 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Embouchure spectaculaire entre océan, lagune et mangrove.</t>
+          <t>Chef-lieu du département du Mono.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Grand-Popo, Mono</t>
+          <t>Lokossa, Mono</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>6.2922216, 1.917286</t>
+          <t>6.6448093, 1.7198215</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2922216,1.917286</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.6448093,1.7198215</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>https://lokossa.mairie.bj/fr/decouverte</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Mono</t>
+          <t>Atacora</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Ville de Lokossa</t>
+          <t>Parc national de la Pendjari</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1831,27 +2081,37 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Chef-lieu du département du Mono.</t>
+          <t>Réserve faunique majeure, safaris et observation de la faune africaine.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Lokossa, Mono</t>
+          <t>Atacora</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>6.6448093, 1.7198215</t>
+          <t>11.2481125, 1.5983959</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.6448093,1.7198215</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.2481125,1.5983959</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Ouvert toute l'année ; safaris recommandés 6h-11h et 16h-tombée de la nuit</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>https://www.african-parks.org/the-parks/pendjari</t>
         </is>
       </c>
     </row>
@@ -1862,11 +2122,11 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Parc national de la Pendjari</t>
+          <t>Villages Tata Somba</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1876,22 +2136,22 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Réserve faunique majeure, safaris et observation de la faune africaine.</t>
+          <t>Habitats traditionnels fortifiés des Batammariba.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Atacora</t>
+          <t>Natitingou/Boukoumbé, Atacora</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>11.2481125, 1.5983959</t>
+          <t>10.3091173, 1.3735244</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=11.2481125,1.5983959</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3091173,1.3735244</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -1907,36 +2167,36 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Villages Tata Somba</t>
+          <t>Cascades de Tanougou</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Site touristique</t>
+          <t>Loisir</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Habitats traditionnels fortifiés des Batammariba.</t>
+          <t>Chutes d'eau et bassins naturels dans les montagnes de l'Atacora.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Natitingou/Boukoumbé, Atacora</t>
+          <t>Tanongou, Atacora</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>10.3091173, 1.3735244</t>
+          <t>10.8121477, 1.4363443</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3091173,1.3735244</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.8121477,1.4363443</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -1952,41 +2212,51 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Cascades de Tanougou</t>
+          <t>Musée régional de Natitingou</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Loisir</t>
+          <t>Site touristique</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Chutes d'eau et bassins naturels dans les montagnes de l'Atacora.</t>
+          <t>Musée sur les traditions socioculturelles de la région.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Tanongou, Atacora</t>
+          <t>Natitingou, Atacora</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>10.8121477, 1.4363443</t>
+          <t>10.3106873, 1.3802711</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.8121477,1.4363443</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3106873,1.3802711</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Lun-Ven 8h30-18h30, Sam-Dim 9h-18h30</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>+229 97 88 10 80</t>
         </is>
       </c>
     </row>
@@ -1997,36 +2267,36 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Musée régional de Natitingou</t>
+          <t>Chaîne de l'Atacora</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Site touristique</t>
+          <t>Loisir</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Musée sur les traditions socioculturelles de la région.</t>
+          <t>Massif montagneux, randonnée et paysages du nord-ouest du Bénin.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Natitingou, Atacora</t>
+          <t>Atacora (zone)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>10.3106873, 1.3802711</t>
+          <t>10.75, 1.5</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3106873,1.3802711</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.75,1.5</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2038,15 +2308,15 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Atacora</t>
+          <t>Borgou/Donga</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Chaîne de l'Atacora</t>
+          <t>Forêt classée de Wari-Maro</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2056,27 +2326,32 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Massif montagneux, randonnée et paysages du nord-ouest du Bénin.</t>
+          <t>Réserve forestière et faunique de la région.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Atacora (zone)</t>
+          <t>Tchaourou, Borgou / Bassila, Donga</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>10.75, 1.5</t>
+          <t>8.9622901, 2.1843285</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.75,1.5</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=8.9622901,2.1843285</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Statut en évolution : fusion annoncée avec la forêt des Monts Kouffé en un nouveau parc national (déc. gouvernementale nov. 2025).</t>
         </is>
       </c>
     </row>
@@ -2087,56 +2362,61 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Forêt classée de Wari-Maro</t>
+          <t>Village de Bassila</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Loisir</t>
+          <t>Site touristique</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Réserve forestière et faunique de la région.</t>
+          <t>Commune forestière du sud de la Donga.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Donga/Collines (zone Wari-Maro)</t>
+          <t>Bassila, Donga</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>8.9622901, 2.1843285</t>
+          <t>9.006393, 1.6639235</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=8.9622901,2.1843285</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.006393,1.6639235</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>+229 23 30 11 76</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Donga</t>
+          <t>Borgou</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Village de Bassila</t>
+          <t>Musée de plein air de Parakou</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2146,27 +2426,42 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Commune forestière du sud de la Donga.</t>
+          <t>Musée d'art et traditions populaires du nord du Bénin.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Bassila, Donga</t>
+          <t>Parakou, Borgou</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>9.006393, 1.6639235</t>
+          <t>9.3279386, 2.6174022</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.006393,1.6639235</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3279386,2.6174022</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Tous les jours 9h-12h et 15h-18h30, sauf jours fériés</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>+229 23 61 05 78</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>https://tourisme.parakou.bj/2024/01/18/musee-plein-air-et-ethnographique/</t>
         </is>
       </c>
     </row>
@@ -2177,41 +2472,56 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Musée de plein air de Parakou</t>
+          <t>Fête de la Gaani</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Site touristique</t>
+          <t>Événement</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Musée d'art et traditions populaires du nord du Bénin.</t>
+          <t>Grande manifestation culturelle annuelle des Batombu.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Parakou, Borgou</t>
+          <t>Nikki, Borgou</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>9.3279386, 2.6174022</t>
+          <t>9.9276076, 3.2167913</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3279386,2.6174022</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.9276076,3.2167913</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>3 jours fin août (ex. 25-27 août 2026)</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>https://gaani.bj</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Anciennement orthographié « Gani » ; deux fiches en doublon fusionnées.</t>
         </is>
       </c>
     </row>
@@ -2222,21 +2532,21 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Fête de la Gani (Nikki)</t>
+          <t>Palais royal de Nikki</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Événement</t>
+          <t>Site touristique</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Grande manifestation culturelle annuelle des Batombu.</t>
+          <t>Capitale historique des Batombu, siège royal.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2246,12 +2556,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>9.9276076, 3.2167913</t>
+          <t>9.9363278, 3.2105884</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.9276076,3.2167913</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.9363278,3.2105884</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2263,15 +2573,15 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Borgou</t>
+          <t>Alibori</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Palais royal de Nikki</t>
+          <t>Parc national du W</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2281,27 +2591,32 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Capitale historique des Batombu, siège royal.</t>
+          <t>Parc transfrontalier Bénin-Niger-Burkina Faso, UNESCO.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Nikki, Borgou</t>
+          <t>Alibori</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>9.9363278, 3.2105884</t>
+          <t>12.0408333, 3.0341667</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.9363278,3.2105884</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=12.0408333,3.0341667</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Ouvert toute l'année</t>
         </is>
       </c>
     </row>
@@ -2312,36 +2627,36 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Parc national du W</t>
+          <t>Fleuve Niger (rives)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Site touristique</t>
+          <t>Loisir</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Parc transfrontalier Bénin-Niger-Burkina Faso, UNESCO.</t>
+          <t>Rives du fleuve Niger, paysages et activités fluviales.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Alibori</t>
+          <t>Malanville, Alibori</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>12.0408333, 3.0341667</t>
+          <t>11.8633332, 3.3842473</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=12.0408333,3.0341667</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.8633332,3.3842473</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2357,36 +2672,36 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Fleuve Niger (rives)</t>
+          <t>Ville de Kandi</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Loisir</t>
+          <t>Site touristique</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Rives du fleuve Niger, paysages et activités fluviales.</t>
+          <t>Chef-lieu du département de l'Alibori.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Malanville, Alibori</t>
+          <t>Kandi, Alibori</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>11.8633332, 3.3842473</t>
+          <t>11.1305191, 2.9325785</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=11.8633332,3.3842473</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.1305191,2.9325785</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2396,47 +2711,9 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Alibori</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Ville de Kandi</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Site touristique</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Chef-lieu du département de l'Alibori.</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>Kandi, Alibori</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>11.1305191, 2.9325785</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=11.1305191,2.9325785</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>Vérifié (Google Places)</t>
         </is>
       </c>
     </row>
@@ -2463,28 +2740,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2496,7 +2772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2550,6 +2826,36 @@
           <t>Statut</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Horaires</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Téléphone</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Site web</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Nb avis</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Remarque</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2592,6 +2898,16 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>+229 53 64 91 65</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://www.beachsandhotel.com</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2634,6 +2950,12 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="L3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="M3" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2676,6 +2998,27 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>+229 95 21 40 40</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://easyhotelsbenin.com</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" t="n">
+        <v>9</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Notes très divergentes selon la plateforme (2/5 TripAdvisor vs retours positifs ailleurs).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2718,6 +3061,16 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>+229 01 54 28 44 44</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://sites.google.com/view/aquamazone229/accueil</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2844,6 +3197,16 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>+229 01 45 46 42 88</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://nativehotels.net</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2886,6 +3249,16 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>+229 96 18 21 94</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Localisation précise : Kpomassè, lac Ahémé (à ~20 min de Ouidah)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2928,6 +3301,11 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Tous les jours 9h-22h</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2970,6 +3348,21 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>24h/24, 7j/7</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>+229 01 66 04 40 12</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://nadalevasiontours.com</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3012,6 +3405,16 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>+229 96 74 06 13</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://www.visit-ganvie-tourism.com</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3054,6 +3457,16 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Format étendu « Vodun Days » sur 2-3 jours (ex. 8-10 janvier 2026)</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://vodundays.bj</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3096,6 +3509,17 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://artresidence.bj</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>5</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3138,6 +3562,17 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>+229 65 00 38 65</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M15" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3264,6 +3699,11 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Marché quotidien, plus animé mercredi et samedi matin</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3348,6 +3788,11 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>En travaux de réhabilitation — accessibilité à vérifier.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3516,6 +3961,17 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>+229 01 55 40 98 78</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>4</v>
+      </c>
+      <c r="M24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3558,6 +4014,17 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>+229 63 13 64 64</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="M25" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3600,11 +4067,22 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>9h-18h (une source indique 8h-17h)</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="M26" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Zou</t>
+          <t>Atlantique/Zou</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -3624,7 +4102,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Zou/Ouémé (zone Lama)</t>
+          <t>Toffo, Atlantique / Zogbodomey, Zou</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -3684,6 +4162,22 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>+229 22 53 08 89</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>https://jecohotels.com</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="M28" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3726,6 +4220,17 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>+229 94 47 21 35</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
+        <v>3</v>
+      </c>
+      <c r="M29" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3768,6 +4273,16 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>https://loubna-hotel.com</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Référencé en ligne sous le nom « Hôtel Loubna Évolution ».</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3810,6 +4325,11 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Site ouvert toute l'année ; pèlerinage vers le 15 août</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3898,7 +4418,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Couffo</t>
+          <t>Mono</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -3908,33 +4428,49 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Hôtel Arnogos</t>
+          <t>Awale Plage</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Hôtel accessible sur la RN2 à Azové.</t>
+          <t>Hôtel-restaurant en bord de plage à Grand-Popo.</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Azové, Couffo</t>
+          <t>Grand-Popo, Mono</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>6.9326883, 1.7079479</t>
+          <t>6.270213, 1.786942</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.9326883,1.7079479</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.270213,1.786942</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>+229 58 01 01 12</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>https://www.hotel-benin-awaleplage.com</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="M34" t="n">
+        <v>137</v>
       </c>
     </row>
     <row r="35">
@@ -3950,12 +4486,12 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Awale Plage</t>
+          <t>ASVA Beach Resort</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Hôtel-restaurant en bord de plage à Grand-Popo.</t>
+          <t>Hôtel proche de la plage, ambiance festive.</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -3965,12 +4501,12 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>6.270213, 1.786942</t>
+          <t>6.2757733, 1.8104271</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.270213,1.786942</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2757733,1.8104271</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -3992,12 +4528,12 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>ASVA Beach Resort</t>
+          <t>Millenium Popo Beach Hôtel</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Hôtel proche de la plage, ambiance festive.</t>
+          <t>Grand complexe hôtelier en bord de mer.</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -4007,18 +4543,29 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>6.2757733, 1.8104271</t>
+          <t>6.2518431, 1.6979677</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2757733,1.8104271</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2518431,1.6979677</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>+229 6860 1111</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
+        <v>2</v>
+      </c>
+      <c r="M36" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="37">
@@ -4027,19 +4574,19 @@
           <t>Mono</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Millenium Popo Beach Hôtel</t>
+          <t>Excursions avec BAKOLO Tours</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Grand complexe hôtelier en bord de mer.</t>
+          <t>Agence locale pour circuits sur mesure dans la région.</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -4049,17 +4596,27 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>6.2518431, 1.6979677</t>
+          <t>6.2772786, 1.8037903</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2518431,1.6979677</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2772786,1.8037903</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>+229 94 69 96 89</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>https://www.bakolotours.com</t>
         </is>
       </c>
     </row>
@@ -4076,12 +4633,12 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Excursions avec BAKOLO Tours</t>
+          <t>Sortie bateau vers la Bouche du Roy</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Agence locale pour circuits sur mesure dans la région.</t>
+          <t>Excursion vers l'embouchure entre océan et lagune.</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -4091,12 +4648,12 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>6.2772786, 1.8037903</t>
+          <t>6.2922216, 1.917286</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2772786,1.8037903</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2922216,1.917286</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -4108,43 +4665,54 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Mono</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Atacora</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Sortie bateau vers la Bouche du Roy</t>
+          <t>Hôtel Bellevue</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Excursion vers l'embouchure entre océan et lagune.</t>
+          <t>Hôtel historique et chaleureux à Natitingou.</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Grand-Popo, Mono</t>
+          <t>Natitingou, Atacora</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>6.2922216, 1.917286</t>
+          <t>10.3059893, 1.3856433</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2922216,1.917286</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3059893,1.3856433</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>+229 23 82 13 36</t>
+        </is>
+      </c>
+      <c r="L39" t="n">
+        <v>4</v>
+      </c>
+      <c r="M39" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="40">
@@ -4160,12 +4728,12 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Hôtel Bellevue</t>
+          <t>Hôtel Tata Somba</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Hôtel historique et chaleureux à Natitingou.</t>
+          <t>Hôtel au pied des collines, proche des villages Tata Somba.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -4175,18 +4743,24 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>10.3059893, 1.3856433</t>
+          <t>10.3091173, 1.3735244</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3059893,1.3856433</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3091173,1.3735244</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="L40" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M40" t="n">
+        <v>217</v>
       </c>
     </row>
     <row r="41">
@@ -4202,12 +4776,12 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Hôtel Tata Somba</t>
+          <t>Hôtel Totora</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Hôtel au pied des collines, proche des villages Tata Somba.</t>
+          <t>Hôtel avec piscine et vue sur les montagnes.</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -4217,18 +4791,34 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>10.3091173, 1.3735244</t>
+          <t>10.3181651, 1.3738271</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3091173,1.3735244</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3181651,1.3738271</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>+229 62 23 62 52</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>https://www.hoteltotora.com</t>
+        </is>
+      </c>
+      <c r="L41" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="M41" t="n">
+        <v>375</v>
       </c>
     </row>
     <row r="42">
@@ -4237,39 +4827,49 @@
           <t>Atacora</t>
         </is>
       </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Hôtel Totora</t>
+          <t>Safari au Parc national de la Pendjari</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Hôtel avec piscine et vue sur les montagnes.</t>
+          <t>Safari guidé pour observer lions, éléphants, hippopotames.</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Natitingou, Atacora</t>
+          <t>Atacora</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>10.3181651, 1.3738271</t>
+          <t>11.2481125, 1.5983959</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3181651,1.3738271</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.2481125,1.5983959</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Créneaux recommandés 6h-11h et 16h-tombée de la nuit</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>https://www.african-parks.org/the-parks/pendjari</t>
         </is>
       </c>
     </row>
@@ -4286,27 +4886,27 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Safari au Parc national de la Pendjari</t>
+          <t>Visite des villages Tata Somba</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Safari guidé pour observer lions, éléphants, hippopotames.</t>
+          <t>Découverte des habitats fortifiés traditionnels.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Atacora</t>
+          <t>Natitingou/Boukoumbé, Atacora</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>11.2481125, 1.5983959</t>
+          <t>10.3091173, 1.3735244</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=11.2481125,1.5983959</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3091173,1.3735244</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -4328,27 +4928,27 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Visite des villages Tata Somba</t>
+          <t>Randonnée aux cascades de Tanougou</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Découverte des habitats fortifiés traditionnels.</t>
+          <t>Baignade et randonnée dans un cadre naturel.</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Natitingou/Boukoumbé, Atacora</t>
+          <t>Tanongou, Atacora</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>10.3091173, 1.3735244</t>
+          <t>10.8121477, 1.4363443</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3091173,1.3735244</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.8121477,1.4363443</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -4360,42 +4960,47 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Atacora</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Donga</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Randonnée aux cascades de Tanougou</t>
+          <t>Motel Du Lac</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Baignade et randonnée dans un cadre naturel.</t>
+          <t>Hôtel familial réputé pour sa cuisine, à Djougou.</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Tanongou, Atacora</t>
+          <t>Djougou, Donga</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>10.8121477, 1.4363443</t>
+          <t>9.6802129, 1.6527047</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.8121477,1.4363443</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.6802129,1.6527047</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>+229 97 54 06 56</t>
         </is>
       </c>
     </row>
@@ -4412,12 +5017,12 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Motel Du Lac</t>
+          <t>Hôtel de la Donga</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Hôtel familial réputé pour sa cuisine, à Djougou.</t>
+          <t>Hôtel simple et pratique à Djougou.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -4427,18 +5032,29 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>9.6802129, 1.6527047</t>
+          <t>9.6997379, 1.6732916</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.6802129,1.6527047</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.6997379,1.6732916</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>+229 23 80 15 72</t>
+        </is>
+      </c>
+      <c r="L46" t="n">
+        <v>3</v>
+      </c>
+      <c r="M46" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="47">
@@ -4454,12 +5070,12 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Hôtel de la Donga</t>
+          <t>Hôtel Cathas</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Hôtel simple et pratique à Djougou.</t>
+          <t>Hôtel accessible au centre de Djougou.</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -4469,54 +5085,59 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>9.6997379, 1.6732916</t>
+          <t>9.6989611, 1.6729295</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.6997379,1.6732916</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.6989611,1.6729295</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>+229 66 03 37 51</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Donga</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+          <t>Borgou/Donga</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Hôtel Cathas</t>
+          <t>Découverte de la Forêt classée de Wari-Maro</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Hôtel accessible au centre de Djougou.</t>
+          <t>Randonnée nature et observation de la faune.</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Djougou, Donga</t>
+          <t>Tchaourou, Borgou / Bassila, Donga</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>9.6989611, 1.6729295</t>
+          <t>8.9622901, 2.1843285</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.6989611,1.6729295</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=8.9622901,2.1843285</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -4528,37 +5149,37 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Donga</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Borgou</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Découverte de la Forêt classée de Wari-Maro</t>
+          <t>Ola Luxury Hôtel</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Randonnée nature et observation de la faune.</t>
+          <t>Hôtel confortable et bien noté à Parakou.</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Zone Wari-Maro, Donga</t>
+          <t>Parakou, Borgou</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>8.9622901, 2.1843285</t>
+          <t>9.3553016, 2.6330228</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=8.9622901,2.1843285</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3553016,2.6330228</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -4580,12 +5201,12 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Ola Luxury Hôtel</t>
+          <t>Kobourou City Hôtel</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Hôtel confortable et bien noté à Parakou.</t>
+          <t>Grand hôtel avec piscine à Parakou.</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -4595,18 +5216,24 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>9.3553016, 2.6330228</t>
+          <t>9.3664096, 2.6247833</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3553016,2.6330228</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3664096,2.6247833</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="L50" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="M50" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="51">
@@ -4622,12 +5249,12 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Kobourou City Hôtel</t>
+          <t>Hôtel Iya-Oasis</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Grand hôtel avec piscine à Parakou.</t>
+          <t>Hôtel au décor traditionnel, très bien noté à Parakou.</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -4637,18 +5264,24 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>9.3664096, 2.6247833</t>
+          <t>9.3457835, 2.6373219</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3664096,2.6247833</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3457835,2.6373219</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="L51" t="n">
+        <v>5</v>
+      </c>
+      <c r="M51" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="52">
@@ -4657,19 +5290,19 @@
           <t>Borgou</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Hôtel Iya-Oasis</t>
+          <t>Visite du musée de plein air de Parakou</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Hôtel au décor traditionnel, très bien noté à Parakou.</t>
+          <t>Découverte de l'art et des traditions du nord du Bénin.</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -4679,54 +5312,69 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>9.3457835, 2.6373219</t>
+          <t>9.3279386, 2.6174022</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3457835,2.6373219</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3279386,2.6174022</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Tous les jours 9h-12h et 15h-18h30, sauf jours fériés</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>+229 23 61 05 78</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>https://tourisme.parakou.bj/2024/01/18/musee-plein-air-et-ethnographique/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Borgou</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Alibori</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Visite du musée de plein air de Parakou</t>
+          <t>Hôtel Séjour du Sahel</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Découverte de l'art et des traditions du nord du Bénin.</t>
+          <t>Hôtel propre et sécurisé à Malanville.</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Parakou, Borgou</t>
+          <t>Malanville, Alibori</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>9.3279386, 2.6174022</t>
+          <t>11.8523034, 3.389122</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3279386,2.6174022</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.8523034,3.389122</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -4738,37 +5386,37 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Borgou</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>Événement</t>
+          <t>Alibori</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Fête de la Gani</t>
+          <t>Safari au Parc national du W</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Grande manifestation culturelle annuelle des Batombu à Nikki.</t>
+          <t>Observation de la faune dans le parc transfrontalier UNESCO.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Nikki, Borgou</t>
+          <t>Alibori</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>9.9276076, 3.2167913</t>
+          <t>12.0408333, 3.0341667</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.9276076,3.2167913</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=12.0408333,3.0341667</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -4776,88 +5424,23 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Créneaux recommandés 6h-11h et 16h-tombée de la nuit</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Alibori</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Hôtel Séjour du Sahel</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>Hôtel propre et sécurisé à Malanville.</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>Malanville, Alibori</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>11.8523034, 3.389122</t>
-        </is>
-      </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G55" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=11.8523034,3.389122</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
-        <is>
-          <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Alibori</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Safari au Parc national du W</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>Observation de la faune dans le parc transfrontalier UNESCO.</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>Alibori</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>12.0408333, 3.0341667</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=12.0408333,3.0341667</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>Vérifié (Google Places)</t>
         </is>
       </c>
     </row>
@@ -4896,29 +5479,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId53"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Retire le contenu événementiel du périmètre produit
Mise à jour de conception : Gosee ne présente pas d'agenda daté. Retire
la catégorie "evenement" du modèle (Category, schema Supabase), les 4
lieux concernés du jeu de données (xlsx source + JSON régénéré), et les
mentions dans l'UI/les métadonnées. CLAUDE.md passe de 7 à 6 piliers
(le pilier "Voir ce qui se passe maintenant" est retiré, la billetterie
devient le pilier 6).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benin_contenu_curation.xlsx
+++ b/benin_contenu_curation.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O43"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1504,61 +1504,56 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Sociétés de masques Guèlèdè, Sakété</t>
+          <t>Ville de Pobè</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Événement</t>
+          <t>Site touristique</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Spectacles traditionnels de masques et danses, patrimoine immatériel UNESCO.</t>
+          <t>Chef-lieu du département du Plateau, culture yoruba-nago.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Sakété, Plateau</t>
+          <t>Pobè, Plateau</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>6.7368274, 2.6636066</t>
+          <t>6.9832415, 2.6636066</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.7368274,2.6636066</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.9832415,2.6636066</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>Patrimoine culturel immatériel (UNESCO) ; le berceau historique documenté est plutôt Kétou/Savè.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Plateau</t>
+          <t>Zou</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Ville de Pobè</t>
+          <t>Palais royaux d'Abomey</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1568,28 +1563,44 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Chef-lieu du département du Plateau, culture yoruba-nago.</t>
+          <t>Ensemble de palais du royaume du Dahomey, classé UNESCO.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Pobè, Plateau</t>
+          <t>Abomey, Zou</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>6.9832415, 2.6636066</t>
+          <t>7.1855024, 1.997943</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.9832415,2.6636066</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1855024,1.997943</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Tous les jours, 9h-18h</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>+229 22 50 03 14</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="N20" t="n">
+        <v>105</v>
       </c>
     </row>
     <row r="21">
@@ -1599,21 +1610,21 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Palais royaux d'Abomey</t>
+          <t>Place Béhanzin (Place Goho)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Site touristique</t>
+          <t>Loisir</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Ensemble de palais du royaume du Dahomey, classé UNESCO.</t>
+          <t>Place centrale avec statue du roi Béhanzin, symbole de résistance.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1623,12 +1634,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>7.1855024, 1.997943</t>
+          <t>7.1842529, 2.0078158</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1855024,1.997943</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1842529,2.0078158</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1636,35 +1647,30 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Tous les jours, 9h-18h</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>+229 22 50 03 14</t>
-        </is>
-      </c>
       <c r="M21" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="N21" t="n">
-        <v>105</v>
+        <v>5</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Un état d'entretien dégradé a été signalé par la presse locale.</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Zou</t>
+          <t>Atlantique/Zou</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Place Béhanzin (Place Goho)</t>
+          <t>Forêt classée de la Lama</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1674,83 +1680,77 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Place centrale avec statue du roi Béhanzin, symbole de résistance.</t>
+          <t>Grande forêt naturelle, observation d'animaux et de flore variée.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Abomey, Zou</t>
+          <t>Toffo, Atlantique / Zogbodomey, Zou</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>7.1842529, 2.0078158</t>
+          <t>6.9179281, 2.1662158</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1842529,2.0078158</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.9179281,2.1662158</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="M22" t="n">
-        <v>4</v>
-      </c>
-      <c r="N22" t="n">
-        <v>5</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>Un état d'entretien dégradé a été signalé par la presse locale.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Atlantique/Zou</t>
+          <t>Collines</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Forêt classée de la Lama</t>
+          <t>Grotte mariale de Dassa-Zoumé</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Loisir</t>
+          <t>Site touristique</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Grande forêt naturelle, observation d'animaux et de flore variée.</t>
+          <t>Lieu de pèlerinage catholique niché dans les collines.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Toffo, Atlantique / Zogbodomey, Zou</t>
+          <t>Dassa-Zoumé, Collines</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>6.9179281, 2.1662158</t>
+          <t>7.7752876, 2.1865136</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.9179281,2.1662158</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.7752876,2.1865136</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Ouvert toute l'année ; grand pèlerinage fin août</t>
         </is>
       </c>
     </row>
@@ -1761,11 +1761,11 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Grotte mariale de Dassa-Zoumé</t>
+          <t>Savalou (ville historique, culte vaudou)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1775,72 +1775,67 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Lieu de pèlerinage catholique niché dans les collines.</t>
+          <t>Ville traditionnelle marquée par la royauté locale et le culte vaudou.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Dassa-Zoumé, Collines</t>
+          <t>Savalou, Collines</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>7.7752876, 2.1865136</t>
+          <t>7.9301365, 1.9710284</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.7752876,2.1865136</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.9301365,1.9710284</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Ouvert toute l'année ; grand pèlerinage fin août</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Collines</t>
+          <t>Mono</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Savalou (ville historique, culte vaudou)</t>
+          <t>Plage de Grand-Popo</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Site touristique</t>
+          <t>Loisir</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Ville traditionnelle marquée par la royauté locale et le culte vaudou.</t>
+          <t>Plage réputée du littoral béninois, tourisme balnéaire.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Savalou, Collines</t>
+          <t>Grand-Popo, Mono</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>7.9301365, 1.9710284</t>
+          <t>6.2639324, 1.7417143</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.9301365,1.9710284</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2639324,1.7417143</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1856,41 +1851,51 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Plage de Grand-Popo</t>
+          <t>Village de Possotomè</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Loisir</t>
+          <t>Site touristique</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Plage réputée du littoral béninois, tourisme balnéaire.</t>
+          <t>Village au bord du lac Ahémé, source d'eau thermale.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Grand-Popo, Mono</t>
+          <t>Possotomè, Bopa, Mono</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>6.2639324, 1.7417143</t>
+          <t>6.520838, 1.9625132</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2639324,1.7417143</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.520838,1.9625132</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>+229 95 28 52 20</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://www.ecobenin.org/possotome</t>
         </is>
       </c>
     </row>
@@ -1901,11 +1906,11 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Village de Possotomè</t>
+          <t>Bouche du Roy</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1915,22 +1920,22 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Village au bord du lac Ahémé, source d'eau thermale.</t>
+          <t>Embouchure spectaculaire entre océan, lagune et mangrove.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Possotomè, Bopa, Mono</t>
+          <t>Grand-Popo, Mono</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>6.520838, 1.9625132</t>
+          <t>6.2922216, 1.917286</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.520838,1.9625132</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2922216,1.917286</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -1940,13 +1945,19 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>+229 95 28 52 20</t>
+          <t>+229 60 63 08 18</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.ecobenin.org/possotome</t>
-        </is>
+          <t>https://www.boucheduroy.bj</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>4</v>
+      </c>
+      <c r="N27" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -1956,11 +1967,11 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Bouche du Roy</t>
+          <t>Ville de Lokossa</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1970,22 +1981,22 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Embouchure spectaculaire entre océan, lagune et mangrove.</t>
+          <t>Chef-lieu du département du Mono.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Grand-Popo, Mono</t>
+          <t>Lokossa, Mono</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>6.2922216, 1.917286</t>
+          <t>6.6448093, 1.7198215</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2922216,1.917286</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.6448093,1.7198215</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -1993,35 +2004,24 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>+229 60 63 08 18</t>
-        </is>
-      </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.boucheduroy.bj</t>
-        </is>
-      </c>
-      <c r="M28" t="n">
-        <v>4</v>
-      </c>
-      <c r="N28" t="n">
-        <v>2</v>
+          <t>https://lokossa.mairie.bj/fr/decouverte</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Mono</t>
+          <t>Atacora</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Ville de Lokossa</t>
+          <t>Parc national de la Pendjari</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -2031,22 +2031,22 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Chef-lieu du département du Mono.</t>
+          <t>Réserve faunique majeure, safaris et observation de la faune africaine.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Lokossa, Mono</t>
+          <t>Atacora</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>6.6448093, 1.7198215</t>
+          <t>11.2481125, 1.5983959</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.6448093,1.7198215</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.2481125,1.5983959</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2054,9 +2054,14 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Ouvert toute l'année ; safaris recommandés 6h-11h et 16h-tombée de la nuit</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://lokossa.mairie.bj/fr/decouverte</t>
+          <t>https://www.african-parks.org/the-parks/pendjari</t>
         </is>
       </c>
     </row>
@@ -2067,11 +2072,11 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Parc national de la Pendjari</t>
+          <t>Villages Tata Somba</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2081,37 +2086,27 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Réserve faunique majeure, safaris et observation de la faune africaine.</t>
+          <t>Habitats traditionnels fortifiés des Batammariba.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Atacora</t>
+          <t>Natitingou/Boukoumbé, Atacora</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>11.2481125, 1.5983959</t>
+          <t>10.3091173, 1.3735244</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=11.2481125,1.5983959</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3091173,1.3735244</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Ouvert toute l'année ; safaris recommandés 6h-11h et 16h-tombée de la nuit</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>https://www.african-parks.org/the-parks/pendjari</t>
         </is>
       </c>
     </row>
@@ -2122,36 +2117,36 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Villages Tata Somba</t>
+          <t>Cascades de Tanougou</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Site touristique</t>
+          <t>Loisir</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Habitats traditionnels fortifiés des Batammariba.</t>
+          <t>Chutes d'eau et bassins naturels dans les montagnes de l'Atacora.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Natitingou/Boukoumbé, Atacora</t>
+          <t>Tanongou, Atacora</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>10.3091173, 1.3735244</t>
+          <t>10.8121477, 1.4363443</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3091173,1.3735244</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.8121477,1.4363443</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2167,41 +2162,51 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Cascades de Tanougou</t>
+          <t>Musée régional de Natitingou</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Loisir</t>
+          <t>Site touristique</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Chutes d'eau et bassins naturels dans les montagnes de l'Atacora.</t>
+          <t>Musée sur les traditions socioculturelles de la région.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Tanongou, Atacora</t>
+          <t>Natitingou, Atacora</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>10.8121477, 1.4363443</t>
+          <t>10.3106873, 1.3802711</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.8121477,1.4363443</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3106873,1.3802711</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Lun-Ven 8h30-18h30, Sam-Dim 9h-18h30</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>+229 97 88 10 80</t>
         </is>
       </c>
     </row>
@@ -2212,66 +2217,56 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Musée régional de Natitingou</t>
+          <t>Chaîne de l'Atacora</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Site touristique</t>
+          <t>Loisir</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Musée sur les traditions socioculturelles de la région.</t>
+          <t>Massif montagneux, randonnée et paysages du nord-ouest du Bénin.</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Natitingou, Atacora</t>
+          <t>Atacora (zone)</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>10.3106873, 1.3802711</t>
+          <t>10.75, 1.5</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3106873,1.3802711</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.75,1.5</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Lun-Ven 8h30-18h30, Sam-Dim 9h-18h30</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>+229 97 88 10 80</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Atacora</t>
+          <t>Borgou/Donga</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Chaîne de l'Atacora</t>
+          <t>Forêt classée de Wari-Maro</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2281,67 +2276,72 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Massif montagneux, randonnée et paysages du nord-ouest du Bénin.</t>
+          <t>Réserve forestière et faunique de la région.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Atacora (zone)</t>
+          <t>Tchaourou, Borgou / Bassila, Donga</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>10.75, 1.5</t>
+          <t>8.9622901, 2.1843285</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.75,1.5</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=8.9622901,2.1843285</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Statut en évolution : fusion annoncée avec la forêt des Monts Kouffé en un nouveau parc national (déc. gouvernementale nov. 2025).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Borgou/Donga</t>
+          <t>Donga</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Forêt classée de Wari-Maro</t>
+          <t>Village de Bassila</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Loisir</t>
+          <t>Site touristique</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Réserve forestière et faunique de la région.</t>
+          <t>Commune forestière du sud de la Donga.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Tchaourou, Borgou / Bassila, Donga</t>
+          <t>Bassila, Donga</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>8.9622901, 2.1843285</t>
+          <t>9.006393, 1.6639235</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=8.9622901,2.1843285</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.006393,1.6639235</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2349,24 +2349,24 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>Statut en évolution : fusion annoncée avec la forêt des Monts Kouffé en un nouveau parc national (déc. gouvernementale nov. 2025).</t>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>+229 23 30 11 76</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Donga</t>
+          <t>Borgou</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Village de Bassila</t>
+          <t>Musée de plein air de Parakou</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2376,22 +2376,22 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Commune forestière du sud de la Donga.</t>
+          <t>Musée d'art et traditions populaires du nord du Bénin.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Bassila, Donga</t>
+          <t>Parakou, Borgou</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>9.006393, 1.6639235</t>
+          <t>9.3279386, 2.6174022</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.006393,1.6639235</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3279386,2.6174022</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2399,9 +2399,19 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Tous les jours 9h-12h et 15h-18h30, sauf jours fériés</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>+229 23 30 11 76</t>
+          <t>+229 23 61 05 78</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://tourisme.parakou.bj/2024/01/18/musee-plein-air-et-ethnographique/</t>
         </is>
       </c>
     </row>
@@ -2412,11 +2422,11 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Musée de plein air de Parakou</t>
+          <t>Palais royal de Nikki</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2426,82 +2436,67 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Musée d'art et traditions populaires du nord du Bénin.</t>
+          <t>Capitale historique des Batombu, siège royal.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Parakou, Borgou</t>
+          <t>Nikki, Borgou</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>9.3279386, 2.6174022</t>
+          <t>9.9363278, 3.2105884</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3279386,2.6174022</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.9363278,3.2105884</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>Tous les jours 9h-12h et 15h-18h30, sauf jours fériés</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>+229 23 61 05 78</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>https://tourisme.parakou.bj/2024/01/18/musee-plein-air-et-ethnographique/</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Borgou</t>
+          <t>Alibori</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Fête de la Gaani</t>
+          <t>Parc national du W</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Événement</t>
+          <t>Site touristique</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Grande manifestation culturelle annuelle des Batombu.</t>
+          <t>Parc transfrontalier Bénin-Niger-Burkina Faso, UNESCO.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Nikki, Borgou</t>
+          <t>Alibori</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>9.9276076, 3.2167913</t>
+          <t>12.0408333, 3.0341667</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.9276076,3.2167913</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=12.0408333,3.0341667</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2511,57 +2506,47 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>3 jours fin août (ex. 25-27 août 2026)</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>https://gaani.bj</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>Anciennement orthographié « Gani » ; deux fiches en doublon fusionnées.</t>
+          <t>Ouvert toute l'année</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Borgou</t>
+          <t>Alibori</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Palais royal de Nikki</t>
+          <t>Fleuve Niger (rives)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Site touristique</t>
+          <t>Loisir</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Capitale historique des Batombu, siège royal.</t>
+          <t>Rives du fleuve Niger, paysages et activités fluviales.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Nikki, Borgou</t>
+          <t>Malanville, Alibori</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>9.9363278, 3.2105884</t>
+          <t>11.8633332, 3.3842473</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.9363278,3.2105884</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.8633332,3.3842473</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2577,11 +2562,11 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Parc national du W</t>
+          <t>Ville de Kandi</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2591,22 +2576,22 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Parc transfrontalier Bénin-Niger-Burkina Faso, UNESCO.</t>
+          <t>Chef-lieu du département de l'Alibori.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Alibori</t>
+          <t>Kandi, Alibori</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>12.0408333, 3.0341667</t>
+          <t>11.1305191, 2.9325785</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=12.0408333,3.0341667</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.1305191,2.9325785</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2614,104 +2599,9 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>Ouvert toute l'année</t>
-        </is>
-      </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Alibori</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Fleuve Niger (rives)</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Loisir</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Rives du fleuve Niger, paysages et activités fluviales.</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>Malanville, Alibori</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>11.8633332, 3.3842473</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=11.8633332,3.3842473</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Alibori</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Ville de Kandi</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Site touristique</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Chef-lieu du département de l'Alibori.</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>Kandi, Alibori</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>11.1305191, 2.9325785</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=11.1305191,2.9325785</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="H43" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=11.1305191,2.9325785</t>
         </is>
@@ -2737,30 +2627,28 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId39"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2772,7 +2660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:N54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3419,37 +3307,37 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Atlantique</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Événement</t>
+          <t>Ouémé</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Fête du Vodun (10 janvier)</t>
+          <t>Art Résidence Hôtel</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Célébration nationale du culte vaudou, grands rassemblements à Ouidah.</t>
+          <t>Hôtel boutique moderne à Porto-Novo.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Ouidah, Atlantique (chaque 10 janvier)</t>
+          <t>Porto-Novo, Ouémé</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>6.3595647, 2.0851368</t>
+          <t>6.4824678, 2.6114132</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.3595647,2.0851368</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.4824678,2.6114132</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -3457,15 +3345,16 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Format étendu « Vodun Days » sur 2-3 jours (ex. 8-10 janvier 2026)</t>
-        </is>
-      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://vodundays.bj</t>
-        </is>
+          <t>https://artresidence.bj</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>5</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -3481,12 +3370,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Art Résidence Hôtel</t>
+          <t>Tour Eiffel Hôtel Bénin</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Hôtel boutique moderne à Porto-Novo.</t>
+          <t>Grand hôtel avec restaurant et piscine à Porto-Novo.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -3496,12 +3385,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>6.4824678, 2.6114132</t>
+          <t>6.4816315, 2.5956944</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.4824678,2.6114132</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.4816315,2.5956944</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -3509,16 +3398,16 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>https://artresidence.bj</t>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>+229 65 00 38 65</t>
         </is>
       </c>
       <c r="L14" t="n">
+        <v>3</v>
+      </c>
+      <c r="M14" t="n">
         <v>5</v>
-      </c>
-      <c r="M14" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -3527,19 +3416,19 @@
           <t>Ouémé</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Tour Eiffel Hôtel Bénin</t>
+          <t>Parc d'attraction Ifè</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Grand hôtel avec restaurant et piscine à Porto-Novo.</t>
+          <t>Parc récréatif familial à Porto-Novo.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -3549,29 +3438,18 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>6.4816315, 2.5956944</t>
+          <t>6.4707072, 2.6095372</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.4816315,2.5956944</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.4707072,2.6095372</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>+229 65 00 38 65</t>
-        </is>
-      </c>
-      <c r="L15" t="n">
-        <v>3</v>
-      </c>
-      <c r="M15" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -3587,27 +3465,27 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Parc d'attraction Ifè</t>
+          <t>Balade sur la Rivière Noire</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Parc récréatif familial à Porto-Novo.</t>
+          <t>Excursion en pirogue sur la Rivière Noire, village d'artisans.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Porto-Novo, Ouémé</t>
+          <t>Adjarra, Ouémé</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>6.4707072, 2.6095372</t>
+          <t>6.5429012, 2.6715489</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.4707072,2.6095372</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.5429012,2.6715489</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -3629,79 +3507,79 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Balade sur la Rivière Noire</t>
+          <t>Visite du Grand Marché de Porto-Novo</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Excursion en pirogue sur la Rivière Noire, village d'artisans.</t>
+          <t>Immersion dans le grand marché local.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Adjarra, Ouémé</t>
+          <t>Porto-Novo, Ouémé</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>6.5429012, 2.6715489</t>
+          <t>6.470905, 2.6266839</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.5429012,2.6715489</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.470905,2.6266839</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Marché quotidien, plus animé mercredi et samedi matin</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Ouémé</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Plateau</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Visite du Grand Marché de Porto-Novo</t>
+          <t>Adebayo Hôtel</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Immersion dans le grand marché local.</t>
+          <t>Hôtel avec restaurant, l'un des mieux notés de Pobè.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Porto-Novo, Ouémé</t>
+          <t>Pobè, Plateau</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>6.470905, 2.6266839</t>
+          <t>6.9774796, 2.658367</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.470905,2.6266839</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.9774796,2.658367</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Marché quotidien, plus animé mercredi et samedi matin</t>
         </is>
       </c>
     </row>
@@ -3711,39 +3589,44 @@
           <t>Plateau</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Adebayo Hôtel</t>
+          <t>Visite du musée Akaba Idena</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Hôtel avec restaurant, l'un des mieux notés de Pobè.</t>
+          <t>Découverte de l'histoire de Kétou et des portes magiques.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Pobè, Plateau</t>
+          <t>Kétou, Plateau</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>6.9774796, 2.658367</t>
+          <t>7.3634919, 2.6016927</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.9774796,2.658367</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.3634919,2.6016927</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>En travaux de réhabilitation — accessibilité à vérifier.</t>
         </is>
       </c>
     </row>
@@ -3760,12 +3643,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Visite du musée Akaba Idena</t>
+          <t>Balade dans la cité royale de Kétou</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Découverte de l'histoire de Kétou et des portes magiques.</t>
+          <t>Immersion dans l'histoire yoruba-nago.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -3775,59 +3658,54 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>7.3634919, 2.6016927</t>
+          <t>7.3603376, 2.6040436</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.3634919,2.6016927</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.3603376,2.6040436</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>En travaux de réhabilitation — accessibilité à vérifier.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Plateau</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Zou</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Balade dans la cité royale de Kétou</t>
+          <t>Ekagnon Hôtel Abomey</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Immersion dans l'histoire yoruba-nago.</t>
+          <t>Hôtel haut de gamme, l'un des mieux notés d'Abomey.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Kétou, Plateau</t>
+          <t>Abomey, Zou</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>7.3603376, 2.6040436</t>
+          <t>7.1640097, 2.0021363</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.3603376,2.6040436</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1640097,2.0021363</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -3839,43 +3717,54 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Plateau</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Événement</t>
+          <t>Zou</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Guèlèdè (spectacle de masques)</t>
+          <t>Bois Vert Hôtel</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Spectacle traditionnel de masques et danses, patrimoine UNESCO, Kétou/Sakété.</t>
+          <t>Hôtel confortable proche du centre d'Abomey.</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Kétou/Sakété, Plateau</t>
+          <t>Abomey, Zou</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>6.7368274, 2.6636066</t>
+          <t>7.1732015, 1.9902517</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.7368274,2.6636066</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1732015,1.9902517</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>+229 01 55 40 98 78</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>4</v>
+      </c>
+      <c r="M22" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -3891,12 +3780,12 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Ekagnon Hôtel Abomey</t>
+          <t>Chez Sabine</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Hôtel haut de gamme, l'un des mieux notés d'Abomey.</t>
+          <t>Maison d'hôtes chaleureuse à Abomey.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -3906,18 +3795,29 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>7.1640097, 2.0021363</t>
+          <t>7.183616, 2.0302333</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1640097,2.0021363</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.183616,2.0302333</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>+229 63 13 64 64</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="M23" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="24">
@@ -3926,19 +3826,19 @@
           <t>Zou</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Bois Vert Hôtel</t>
+          <t>Visite guidée des palais royaux (Guide Abomey)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Hôtel confortable proche du centre d'Abomey.</t>
+          <t>Guide local pour explorer l'histoire du royaume du Dahomey.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -3948,12 +3848,12 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>7.1732015, 1.9902517</t>
+          <t>7.1889261, 1.9942085</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1732015,1.9902517</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1889261,1.9942085</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -3961,105 +3861,94 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>+229 01 55 40 98 78</t>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>9h-18h (une source indique 8h-17h)</t>
         </is>
       </c>
       <c r="L24" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="M24" t="n">
-        <v>3</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Zou</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+          <t>Atlantique/Zou</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Chez Sabine</t>
+          <t>Découverte de la Forêt classée de la Lama</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Maison d'hôtes chaleureuse à Abomey.</t>
+          <t>Observation de la faune et de la flore.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Abomey, Zou</t>
+          <t>Toffo, Atlantique / Zogbodomey, Zou</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>7.183616, 2.0302333</t>
+          <t>6.9179281, 2.1662158</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.183616,2.0302333</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.9179281,2.1662158</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>+229 63 13 64 64</t>
-        </is>
-      </c>
-      <c r="L25" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="M25" t="n">
-        <v>30</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Zou</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Collines</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Visite guidée des palais royaux (Guide Abomey)</t>
+          <t>Hôtel Jeco</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Guide local pour explorer l'histoire du royaume du Dahomey.</t>
+          <t>Hôtel confortable avec piscine à Dassa-Zoumé.</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Abomey, Zou</t>
+          <t>Dassa-Zoumé, Collines</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>7.1889261, 1.9942085</t>
+          <t>7.7790481, 2.1843505</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.1889261,1.9942085</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.7790481,2.1843505</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -4067,58 +3956,74 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>9h-18h (une source indique 8h-17h)</t>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>+229 22 53 08 89</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>https://jecohotels.com</t>
         </is>
       </c>
       <c r="L26" t="n">
-        <v>3.7</v>
+        <v>2.6</v>
       </c>
       <c r="M26" t="n">
-        <v>105</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Atlantique/Zou</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Collines</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Découverte de la Forêt classée de la Lama</t>
+          <t>Auberge de Dassa-Zoumé</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Observation de la faune et de la flore.</t>
+          <t>Auberge bien située, halte pratique sur la route du nord.</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Toffo, Atlantique / Zogbodomey, Zou</t>
+          <t>Dassa-Zoumé, Collines</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>6.9179281, 2.1662158</t>
+          <t>7.7811209, 2.1824554</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.9179281,2.1662158</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.7811209,2.1824554</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>+229 94 47 21 35</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
+        <v>3</v>
+      </c>
+      <c r="M27" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="28">
@@ -4134,27 +4039,27 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Hôtel Jeco</t>
+          <t>Loubna Hôtel &amp; Restauration</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Hôtel confortable avec piscine à Dassa-Zoumé.</t>
+          <t>Hôtel confortable à Paouignan, près des collines.</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Dassa-Zoumé, Collines</t>
+          <t>Paouignan, Collines</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>7.7790481, 2.1843505</t>
+          <t>7.6698299, 2.2237021</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.7790481,2.1843505</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.6698299,2.2237021</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -4162,21 +4067,15 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>+229 22 53 08 89</t>
-        </is>
-      </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>https://jecohotels.com</t>
-        </is>
-      </c>
-      <c r="L28" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="M28" t="n">
-        <v>43</v>
+          <t>https://loubna-hotel.com</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Référencé en ligne sous le nom « Hôtel Loubna Évolution ».</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -4185,19 +4084,19 @@
           <t>Collines</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Auberge de Dassa-Zoumé</t>
+          <t>Pèlerinage à la Grotte mariale de Dassa</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Auberge bien située, halte pratique sur la route du nord.</t>
+          <t>Visite du site de pèlerinage catholique niché dans les collines.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -4207,12 +4106,12 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>7.7811209, 2.1824554</t>
+          <t>7.7752876, 2.1865136</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.7811209,2.1824554</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.7752876,2.1865136</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -4220,16 +4119,10 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>+229 94 47 21 35</t>
-        </is>
-      </c>
-      <c r="L29" t="n">
-        <v>3</v>
-      </c>
-      <c r="M29" t="n">
-        <v>12</v>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Site ouvert toute l'année ; pèlerinage vers le 15 août</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -4238,49 +4131,39 @@
           <t>Collines</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Loubna Hôtel &amp; Restauration</t>
+          <t>Visite du sanctuaire vaudou de Dankoli</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Hôtel confortable à Paouignan, près des collines.</t>
+          <t>Découverte d'un des sanctuaires vaudou les plus actifs d'Afrique de l'Ouest.</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Paouignan, Collines</t>
+          <t>Savalou, Collines</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>7.6698299, 2.2237021</t>
+          <t>7.9301365, 1.9710284</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.6698299,2.2237021</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.9301365,1.9710284</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>https://loubna-hotel.com</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>Référencé en ligne sous le nom « Hôtel Loubna Évolution ».</t>
         </is>
       </c>
     </row>
@@ -4297,116 +4180,127 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Pèlerinage à la Grotte mariale de Dassa</t>
+          <t>Visite du Palais Royal de Savalou</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Visite du site de pèlerinage catholique niché dans les collines.</t>
+          <t>Immersion dans l'histoire du royaume Mahi.</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Dassa-Zoumé, Collines</t>
+          <t>Savalou, Collines</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>7.7752876, 2.1865136</t>
+          <t>7.9313702, 1.9726773</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.7752876,2.1865136</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=7.9313702,1.9726773</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Site ouvert toute l'année ; pèlerinage vers le 15 août</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Collines</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Mono</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Visite du sanctuaire vaudou de Dankoli</t>
+          <t>Awale Plage</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Découverte d'un des sanctuaires vaudou les plus actifs d'Afrique de l'Ouest.</t>
+          <t>Hôtel-restaurant en bord de plage à Grand-Popo.</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Savalou, Collines</t>
+          <t>Grand-Popo, Mono</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>7.9301365, 1.9710284</t>
+          <t>6.270213, 1.786942</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.9301365,1.9710284</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.270213,1.786942</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>+229 58 01 01 12</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>https://www.hotel-benin-awaleplage.com</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="M32" t="n">
+        <v>137</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Collines</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Mono</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Visite du Palais Royal de Savalou</t>
+          <t>ASVA Beach Resort</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Immersion dans l'histoire du royaume Mahi.</t>
+          <t>Hôtel proche de la plage, ambiance festive.</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Savalou, Collines</t>
+          <t>Grand-Popo, Mono</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>7.9313702, 1.9726773</t>
+          <t>6.2757733, 1.8104271</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=7.9313702,1.9726773</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2757733,1.8104271</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -4428,12 +4322,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Awale Plage</t>
+          <t>Millenium Popo Beach Hôtel</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Hôtel-restaurant en bord de plage à Grand-Popo.</t>
+          <t>Grand complexe hôtelier en bord de mer.</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -4443,12 +4337,12 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>6.270213, 1.786942</t>
+          <t>6.2518431, 1.6979677</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.270213,1.786942</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2518431,1.6979677</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -4458,19 +4352,14 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>+229 58 01 01 12</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>https://www.hotel-benin-awaleplage.com</t>
+          <t>+229 6860 1111</t>
         </is>
       </c>
       <c r="L34" t="n">
-        <v>3.6</v>
+        <v>2</v>
       </c>
       <c r="M34" t="n">
-        <v>137</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35">
@@ -4479,19 +4368,19 @@
           <t>Mono</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>ASVA Beach Resort</t>
+          <t>Excursions avec BAKOLO Tours</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Hôtel proche de la plage, ambiance festive.</t>
+          <t>Agence locale pour circuits sur mesure dans la région.</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -4501,17 +4390,27 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>6.2757733, 1.8104271</t>
+          <t>6.2772786, 1.8037903</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2757733,1.8104271</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2772786,1.8037903</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>+229 94 69 96 89</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>https://www.bakolotours.com</t>
         </is>
       </c>
     </row>
@@ -4521,19 +4420,19 @@
           <t>Mono</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Millenium Popo Beach Hôtel</t>
+          <t>Sortie bateau vers la Bouche du Roy</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Grand complexe hôtelier en bord de mer.</t>
+          <t>Excursion vers l'embouchure entre océan et lagune.</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -4543,65 +4442,54 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>6.2518431, 1.6979677</t>
+          <t>6.2922216, 1.917286</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2518431,1.6979677</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2922216,1.917286</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>+229 6860 1111</t>
-        </is>
-      </c>
-      <c r="L36" t="n">
-        <v>2</v>
-      </c>
-      <c r="M36" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Mono</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Atacora</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Excursions avec BAKOLO Tours</t>
+          <t>Hôtel Bellevue</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Agence locale pour circuits sur mesure dans la région.</t>
+          <t>Hôtel historique et chaleureux à Natitingou.</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Grand-Popo, Mono</t>
+          <t>Natitingou, Atacora</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>6.2772786, 1.8037903</t>
+          <t>10.3059893, 1.3856433</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2772786,1.8037903</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3059893,1.3856433</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -4611,55 +4499,62 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>+229 94 69 96 89</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>https://www.bakolotours.com</t>
-        </is>
+          <t>+229 23 82 13 36</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
+        <v>4</v>
+      </c>
+      <c r="M37" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Mono</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Atacora</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Sortie bateau vers la Bouche du Roy</t>
+          <t>Hôtel Tata Somba</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Excursion vers l'embouchure entre océan et lagune.</t>
+          <t>Hôtel au pied des collines, proche des villages Tata Somba.</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Grand-Popo, Mono</t>
+          <t>Natitingou, Atacora</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>6.2922216, 1.917286</t>
+          <t>10.3091173, 1.3735244</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=6.2922216,1.917286</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3091173,1.3735244</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="L38" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M38" t="n">
+        <v>217</v>
       </c>
     </row>
     <row r="39">
@@ -4675,12 +4570,12 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Hôtel Bellevue</t>
+          <t>Hôtel Totora</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Hôtel historique et chaleureux à Natitingou.</t>
+          <t>Hôtel avec piscine et vue sur les montagnes.</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -4690,12 +4585,12 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>10.3059893, 1.3856433</t>
+          <t>10.3181651, 1.3738271</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3059893,1.3856433</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3181651,1.3738271</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -4705,14 +4600,19 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>+229 23 82 13 36</t>
+          <t>+229 62 23 62 52</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>https://www.hoteltotora.com</t>
         </is>
       </c>
       <c r="L39" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="M39" t="n">
-        <v>20</v>
+        <v>375</v>
       </c>
     </row>
     <row r="40">
@@ -4721,34 +4621,34 @@
           <t>Atacora</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Hôtel Tata Somba</t>
+          <t>Safari au Parc national de la Pendjari</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Hôtel au pied des collines, proche des villages Tata Somba.</t>
+          <t>Safari guidé pour observer lions, éléphants, hippopotames.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Natitingou, Atacora</t>
+          <t>Atacora</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>10.3091173, 1.3735244</t>
+          <t>11.2481125, 1.5983959</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3091173,1.3735244</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.2481125,1.5983959</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -4756,11 +4656,15 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
-      <c r="L40" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="M40" t="n">
-        <v>217</v>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Créneaux recommandés 6h-11h et 16h-tombée de la nuit</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>https://www.african-parks.org/the-parks/pendjari</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -4769,56 +4673,40 @@
           <t>Atacora</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Hôtel Totora</t>
+          <t>Visite des villages Tata Somba</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Hôtel avec piscine et vue sur les montagnes.</t>
+          <t>Découverte des habitats fortifiés traditionnels.</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Natitingou, Atacora</t>
+          <t>Natitingou/Boukoumbé, Atacora</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>10.3181651, 1.3738271</t>
+          <t>10.3091173, 1.3735244</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3181651,1.3738271</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3091173,1.3735244</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>+229 62 23 62 52</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>https://www.hoteltotora.com</t>
-        </is>
-      </c>
-      <c r="L41" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="M41" t="n">
-        <v>375</v>
       </c>
     </row>
     <row r="42">
@@ -4834,127 +4722,133 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Safari au Parc national de la Pendjari</t>
+          <t>Randonnée aux cascades de Tanougou</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Safari guidé pour observer lions, éléphants, hippopotames.</t>
+          <t>Baignade et randonnée dans un cadre naturel.</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Atacora</t>
+          <t>Tanongou, Atacora</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>11.2481125, 1.5983959</t>
+          <t>10.8121477, 1.4363443</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=11.2481125,1.5983959</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=10.8121477,1.4363443</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Créneaux recommandés 6h-11h et 16h-tombée de la nuit</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>https://www.african-parks.org/the-parks/pendjari</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Atacora</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Donga</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Visite des villages Tata Somba</t>
+          <t>Motel Du Lac</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Découverte des habitats fortifiés traditionnels.</t>
+          <t>Hôtel familial réputé pour sa cuisine, à Djougou.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Natitingou/Boukoumbé, Atacora</t>
+          <t>Djougou, Donga</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>10.3091173, 1.3735244</t>
+          <t>9.6802129, 1.6527047</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.3091173,1.3735244</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.6802129,1.6527047</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>+229 97 54 06 56</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Atacora</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Donga</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Randonnée aux cascades de Tanougou</t>
+          <t>Hôtel de la Donga</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Baignade et randonnée dans un cadre naturel.</t>
+          <t>Hôtel simple et pratique à Djougou.</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Tanongou, Atacora</t>
+          <t>Djougou, Donga</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>10.8121477, 1.4363443</t>
+          <t>9.6997379, 1.6732916</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=10.8121477,1.4363443</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.6997379,1.6732916</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>+229 23 80 15 72</t>
+        </is>
+      </c>
+      <c r="L44" t="n">
+        <v>3</v>
+      </c>
+      <c r="M44" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="45">
@@ -4970,12 +4864,12 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Motel Du Lac</t>
+          <t>Hôtel Cathas</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Hôtel familial réputé pour sa cuisine, à Djougou.</t>
+          <t>Hôtel accessible au centre de Djougou.</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -4985,12 +4879,12 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>9.6802129, 1.6527047</t>
+          <t>9.6989611, 1.6729295</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.6802129,1.6527047</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.6989611,1.6729295</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -5000,67 +4894,56 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>+229 97 54 06 56</t>
+          <t>+229 66 03 37 51</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Donga</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+          <t>Borgou/Donga</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Hôtel de la Donga</t>
+          <t>Découverte de la Forêt classée de Wari-Maro</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Hôtel simple et pratique à Djougou.</t>
+          <t>Randonnée nature et observation de la faune.</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Djougou, Donga</t>
+          <t>Tchaourou, Borgou / Bassila, Donga</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>9.6997379, 1.6732916</t>
+          <t>8.9622901, 2.1843285</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.6997379,1.6732916</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=8.9622901,2.1843285</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>+229 23 80 15 72</t>
-        </is>
-      </c>
-      <c r="L46" t="n">
-        <v>3</v>
-      </c>
-      <c r="M46" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Donga</t>
+          <t>Borgou</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -5070,80 +4953,81 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Hôtel Cathas</t>
+          <t>Ola Luxury Hôtel</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Hôtel accessible au centre de Djougou.</t>
+          <t>Hôtel confortable et bien noté à Parakou.</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Djougou, Donga</t>
+          <t>Parakou, Borgou</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>9.6989611, 1.6729295</t>
+          <t>9.3553016, 2.6330228</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.6989611,1.6729295</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3553016,2.6330228</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>+229 66 03 37 51</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Borgou/Donga</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
+          <t>Borgou</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Hôtel</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Découverte de la Forêt classée de Wari-Maro</t>
+          <t>Kobourou City Hôtel</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Randonnée nature et observation de la faune.</t>
+          <t>Grand hôtel avec piscine à Parakou.</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Tchaourou, Borgou / Bassila, Donga</t>
+          <t>Parakou, Borgou</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>8.9622901, 2.1843285</t>
+          <t>9.3664096, 2.6247833</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=8.9622901,2.1843285</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3664096,2.6247833</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="L48" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="M48" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="49">
@@ -5159,12 +5043,12 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Ola Luxury Hôtel</t>
+          <t>Hôtel Iya-Oasis</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Hôtel confortable et bien noté à Parakou.</t>
+          <t>Hôtel au décor traditionnel, très bien noté à Parakou.</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -5174,18 +5058,24 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>9.3553016, 2.6330228</t>
+          <t>9.3457835, 2.6373219</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3553016,2.6330228</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3457835,2.6373219</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
+      </c>
+      <c r="L49" t="n">
+        <v>5</v>
+      </c>
+      <c r="M49" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -5194,19 +5084,19 @@
           <t>Borgou</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Activité</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Kobourou City Hôtel</t>
+          <t>Visite du musée de plein air de Parakou</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Grand hôtel avec piscine à Parakou.</t>
+          <t>Découverte de l'art et des traditions du nord du Bénin.</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -5216,12 +5106,12 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>9.3664096, 2.6247833</t>
+          <t>9.3279386, 2.6174022</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3664096,2.6247833</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3279386,2.6174022</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -5229,17 +5119,26 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
-      <c r="L50" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="M50" t="n">
-        <v>6</v>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Tous les jours 9h-12h et 15h-18h30, sauf jours fériés</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>+229 23 61 05 78</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>https://tourisme.parakou.bj/2024/01/18/musee-plein-air-et-ethnographique/</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Borgou</t>
+          <t>Alibori</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -5249,45 +5148,39 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Hôtel Iya-Oasis</t>
+          <t>Hôtel Séjour du Sahel</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Hôtel au décor traditionnel, très bien noté à Parakou.</t>
+          <t>Hôtel propre et sécurisé à Malanville.</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Parakou, Borgou</t>
+          <t>Malanville, Alibori</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>9.3457835, 2.6373219</t>
+          <t>11.8523034, 3.389122</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3457835,2.6373219</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.8523034,3.389122</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Vérifié (Google Places)</t>
         </is>
-      </c>
-      <c r="L51" t="n">
-        <v>5</v>
-      </c>
-      <c r="M51" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Borgou</t>
+          <t>Alibori</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
@@ -5297,27 +5190,27 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Visite du musée de plein air de Parakou</t>
+          <t>Safari au Parc national du W</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Découverte de l'art et des traditions du nord du Bénin.</t>
+          <t>Observation de la faune dans le parc transfrontalier UNESCO.</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Parakou, Borgou</t>
+          <t>Alibori</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>9.3279386, 2.6174022</t>
+          <t>12.0408333, 3.0341667</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=9.3279386,2.6174022</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=12.0408333,3.0341667</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -5327,118 +5220,19 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Tous les jours 9h-12h et 15h-18h30, sauf jours fériés</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>+229 23 61 05 78</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>https://tourisme.parakou.bj/2024/01/18/musee-plein-air-et-ethnographique/</t>
+          <t>Créneaux recommandés 6h-11h et 16h-tombée de la nuit</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>Alibori</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>Hôtel</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Hôtel Séjour du Sahel</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>Hôtel propre et sécurisé à Malanville.</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Malanville, Alibori</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>11.8523034, 3.389122</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=11.8523034,3.389122</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Alibori</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>Activité</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Safari au Parc national du W</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>Observation de la faune dans le parc transfrontalier UNESCO.</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Alibori</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>12.0408333, 3.0341667</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=12.0408333,3.0341667</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>Vérifié (Google Places)</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>Créneaux recommandés 6h-11h et 16h-tombée de la nuit</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=11.8523034,3.389122</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="G56" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=12.0408333,3.0341667</t>
         </is>
@@ -5458,48 +5252,46 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId51"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Infos pratiques des 90 lieux : prix, durée, ambiances, public idéal
Prépare le pilier Recommandations personnalisées : le moteur a besoin de
savoir combien coûte un lieu, combien de temps il demande et à qui il
convient, ce qu'aucun lieu ne renseignait.

Prix sourcés par recherche web quand un tarif public existe (souvent
anciens, signalés comme tels) ; sinon gamme et durée estimées, marquées
infos_estimees et signalées sur la fiche plutôt que présentées comme
vérifiées. Le xlsx reste la source de vérité (6 nouvelles colonnes).

Nécessite d'exécuter la migration de supabase/schema.sql puis npm run
seed pour apparaître en prod ; la fiche masque le bloc tant que les
colonnes sont absentes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRtuV2T5j4ZnKKUy5a7yX4
</commit_message>
<xml_diff>
--- a/benin_contenu_curation.xlsx
+++ b/benin_contenu_curation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="60 Lieux incontournables" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hôtels-Activités-Événements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="60 Lieux incontournables" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Hôtels-Activités-Événements" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'60 Lieux incontournables'!$A$1:$I$43</definedName>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:U43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -579,6 +579,36 @@
           <t>Remarque</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Prix</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Gamme de prix</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Durée</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Ambiances</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Idéal pour</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Infos estimées</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -624,6 +654,36 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Entrée libre (lieu de culte)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>spiritualite, culture</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -690,6 +750,36 @@
       <c r="N3" t="n">
         <v>88</v>
       </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Entrée gratuite</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>art, culture</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -741,6 +831,36 @@
       <c r="N4" t="n">
         <v>72</v>
       </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Accès libre</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>plage, detente</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -792,6 +912,36 @@
       <c r="N5" t="n">
         <v>15</v>
       </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Accès libre (espace public)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>histoire, culture</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -848,6 +998,31 @@
       <c r="N6" t="n">
         <v>15</v>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>sport</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>amis, famille</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -904,6 +1079,36 @@
       <c r="N7" t="n">
         <v>5</v>
       </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Parcours en accès libre ; guide en option</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>histoire, culture</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -965,6 +1170,36 @@
       <c r="N8" t="n">
         <v>142</v>
       </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>≈ 2 000 FCFA / pers. (tarif relevé en 2021)</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>spiritualite, culture</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1016,6 +1251,36 @@
       <c r="N9" t="n">
         <v>10</v>
       </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>≈ 1 100 FCFA / pers. (tarif relevé en 2021)</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>spiritualite, nature, culture</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1077,6 +1342,36 @@
           <t>Possiblement fermé pour rénovation depuis 2026 — vérifier avant de s'y rendre.</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>≈ 5 000 FCFA / pers. pour le musée d'histoire (tarif 2021, fermeture possible)</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>histoire, culture</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1128,6 +1423,36 @@
       <c r="N11" t="n">
         <v>69</v>
       </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>≈ 5 000 à 10 500 FCFA / pers. (pirogue + guide, selon taille du groupe)</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>culture, aventure</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1179,6 +1504,36 @@
       <c r="N12" t="n">
         <v>21</v>
       </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>≈ 1 000 FCFA / pers.</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>histoire, culture</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1235,6 +1590,31 @@
       <c r="N13" t="n">
         <v>21</v>
       </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>histoire, culture, art</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1291,6 +1671,31 @@
       <c r="N14" t="n">
         <v>29</v>
       </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>culture, art</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1351,6 +1756,36 @@
           <t>https://songhai.org</t>
         </is>
       </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Visite guidée d'environ 1 h ; restaurant sur place (≈ 1 200 à 3 500 FCFA le plat)</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>nature, culture</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1401,6 +1836,36 @@
           <t>Messes semaine 6h, 12h45, 18h ; dimanche 7h, 9h, 10h30, 19h</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Entrée libre (lieu de culte)</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>spiritualite, histoire</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1446,6 +1911,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>histoire, culture</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1496,6 +1986,31 @@
           <t>En travaux de réhabilitation — accessibilité à vérifier.</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>histoire, culture</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1541,6 +2056,36 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Découverte libre de la ville</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>culture</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>solo, couple, amis</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1602,6 +2147,36 @@
       <c r="N20" t="n">
         <v>105</v>
       </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>≈ 3 000 à 5 000 FCFA / pers.</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>histoire, culture</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1658,6 +2233,36 @@
           <t>Un état d'entretien dégradé a été signalé par la presse locale.</t>
         </is>
       </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Accès libre (espace public)</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>histoire</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1703,6 +2308,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>journee</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>nature, faune, aventure</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>amis, famille</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1753,6 +2383,36 @@
           <t>Ouvert toute l'année ; grand pèlerinage fin août</t>
         </is>
       </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Accès libre (lieu de pèlerinage)</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>spiritualite, nature</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1798,6 +2458,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>culture, spiritualite, histoire</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>solo, couple, amis</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1843,6 +2528,36 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Accès libre</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>plage, detente</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1898,6 +2613,31 @@
           <t>https://www.ecobenin.org/possotome</t>
         </is>
       </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>nature, detente, culture</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1959,6 +2699,36 @@
       <c r="N27" t="n">
         <v>2</v>
       </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>≈ 10 000 FCFA / pers. en pirogue (réductions possibles en groupe)</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>nature, aventure, plage</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2009,6 +2779,36 @@
           <t>https://lokossa.mairie.bj/fr/decouverte</t>
         </is>
       </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Découverte libre de la ville</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>culture</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>solo, couple, amis</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2064,6 +2864,36 @@
           <t>https://www.african-parks.org/the-parks/pendjari</t>
         </is>
       </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Entrée ≈ 19 € adulte étranger, ≈ 7 € résident béninois (anciens tarifs), + véhicule et guide</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>eleve</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>faune, nature, aventure</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2109,6 +2939,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>culture, histoire</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2154,6 +3009,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>nature, aventure, detente</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2209,6 +3089,31 @@
           <t>+229 97 88 10 80</t>
         </is>
       </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>culture, histoire</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2254,6 +3159,36 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Accès libre ; guide conseillé pour la randonnée</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>journee</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>nature, aventure, sport</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>solo, amis</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2304,6 +3239,31 @@
           <t>Statut en évolution : fusion annoncée avec la forêt des Monts Kouffé en un nouveau parc national (déc. gouvernementale nov. 2025).</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>journee</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>nature, faune, aventure</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>amis</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2354,6 +3314,36 @@
           <t>+229 23 30 11 76</t>
         </is>
       </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Découverte libre</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>nature, culture</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>solo, amis</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2414,6 +3404,31 @@
           <t>https://tourisme.parakou.bj/2024/01/18/musee-plein-air-et-ethnographique/</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>culture, art</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2459,6 +3474,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>histoire, culture</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2509,6 +3549,36 @@
           <t>Ouvert toute l'année</t>
         </is>
       </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Entrée ≈ 10 000 FCFA / 24 h, + véhicule (≈ 60 000 à 70 000 FCFA), guide (≈ 20 000 FCFA) et carburant</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>eleve</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>faune, nature, aventure</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2554,6 +3624,36 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Accès libre ; balade en pirogue à négocier sur place</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>nature, detente</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>solo, couple, amis</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2599,9 +3699,53 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Découverte libre de la ville</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>culture</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>solo, amis</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="H41" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.1305191,2.9325785</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.8633332,3.3842473</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="H43" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=11.1305191,2.9325785</t>
         </is>
@@ -2660,7 +3804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N54"/>
+  <dimension ref="A1:T56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2744,6 +3888,36 @@
           <t>Remarque</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Prix</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Gamme de prix</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Durée</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Ambiances</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Idéal pour</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Infos estimées</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2796,6 +3970,36 @@
           <t>https://www.beachsandhotel.com</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Dès ≈ 33 USD / nuit (plateformes de réservation)</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>detente, plage</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>couple, famille</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2844,6 +4048,36 @@
       <c r="M3" t="n">
         <v>8</v>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Dès ≈ 36 € / nuit (plateformes de réservation)</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>solo, couple</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2907,6 +4141,36 @@
           <t>Notes très divergentes selon la plateforme (2/5 TripAdvisor vs retours positifs ailleurs).</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Dès ≈ 30 USD / nuit (plateformes de réservation)</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>plage, detente</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>solo, couple, amis</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2959,6 +4223,31 @@
           <t>https://sites.google.com/view/aquamazone229/accueil</t>
         </is>
       </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>sport, aventure, plage</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>amis, famille</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3001,6 +4290,36 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Balade libre (transport à prévoir)</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>plage, detente, nature</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3043,6 +4362,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>solo, couple</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3095,6 +4439,36 @@
           <t>https://nativehotels.net</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Dès ≈ 127 £ / nuit (plateformes de réservation)</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>eleve</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>detente, histoire</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>couple</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3147,6 +4521,31 @@
           <t>Localisation précise : Kpomassè, lac Ahémé (à ~20 min de Ouidah)</t>
         </is>
       </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>detente, nature</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>couple, famille</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3194,6 +4593,31 @@
           <t>Tous les jours 9h-22h</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>loisirs</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>amis, famille</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3251,6 +4675,31 @@
           <t>https://nadalevasiontours.com</t>
         </is>
       </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>journee</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>histoire, culture, spiritualite</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3303,6 +4752,36 @@
           <t>https://www.visit-ganvie-tourism.com</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>≈ 5 000 à 10 500 FCFA / pers. (pirogue + guide, selon taille du groupe)</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>culture, aventure</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3356,6 +4835,36 @@
       <c r="M13" t="n">
         <v>1</v>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Dès ≈ 150 USD / nuit (plateformes de réservation)</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>eleve</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>detente, art</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>couple</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3409,6 +4918,36 @@
       <c r="M14" t="n">
         <v>5</v>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Dès ≈ 44 USD / nuit (plateformes de réservation)</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3451,6 +4990,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>loisirs</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>amis, famille</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3493,6 +5057,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>nature, aventure, culture</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3540,6 +5129,36 @@
           <t>Marché quotidien, plus animé mercredi et samedi matin</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Entrée libre (achats en sus)</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>marche, culture</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>solo, couple, amis</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3582,6 +5201,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>solo, couple</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -3629,6 +5273,31 @@
           <t>En travaux de réhabilitation — accessibilité à vérifier.</t>
         </is>
       </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>histoire, culture</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3671,6 +5340,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>histoire, culture</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3713,6 +5407,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>couple, famille</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3766,6 +5485,31 @@
       <c r="M22" t="n">
         <v>3</v>
       </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>solo, couple</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3819,6 +5563,36 @@
       <c r="M23" t="n">
         <v>30</v>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>≈ 34 à 73 USD / nuit pour 2 adultes (plateformes de réservation)</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>detente, culture</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>solo, couple</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3872,6 +5646,36 @@
       <c r="M24" t="n">
         <v>105</v>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Entrée du site ≈ 3 000 à 5 000 FCFA / pers., guide en sus</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>histoire, culture</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3914,6 +5718,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>journee</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>nature, faune, aventure</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>amis, famille</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3972,6 +5801,31 @@
       <c r="M26" t="n">
         <v>43</v>
       </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>couple, famille</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -4025,6 +5879,31 @@
       <c r="M27" t="n">
         <v>12</v>
       </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>solo, amis</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4077,6 +5956,31 @@
           <t>Référencé en ligne sous le nom « Hôtel Loubna Évolution ».</t>
         </is>
       </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>solo, couple</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4124,6 +6028,36 @@
           <t>Site ouvert toute l'année ; pèlerinage vers le 15 août</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Accès libre (lieu de pèlerinage)</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>gratuit</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>spiritualite, nature</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4166,6 +6100,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>spiritualite, culture</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>solo, couple, amis</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4208,6 +6167,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>histoire, culture</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4266,6 +6250,36 @@
       <c r="M32" t="n">
         <v>137</v>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Dès ≈ 29 USD / nuit (plateformes de réservation)</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>plage, detente</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4308,6 +6322,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>plage, detente</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>amis, couple</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4361,6 +6400,31 @@
       <c r="M34" t="n">
         <v>16</v>
       </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>plage, detente</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>couple, famille</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4413,6 +6477,31 @@
           <t>https://www.bakolotours.com</t>
         </is>
       </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>journee</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>nature, culture, aventure</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -4455,6 +6544,36 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>≈ 10 000 FCFA / pers. (réductions possibles en groupe)</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>nature, aventure, plage</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -4508,6 +6627,31 @@
       <c r="M37" t="n">
         <v>20</v>
       </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>solo, couple</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -4556,6 +6700,31 @@
       <c r="M38" t="n">
         <v>217</v>
       </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>detente, culture</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -4614,6 +6783,31 @@
       <c r="M39" t="n">
         <v>375</v>
       </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>detente, nature</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>couple, famille</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -4666,6 +6860,36 @@
           <t>https://www.african-parks.org/the-parks/pendjari</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Entrée ≈ 19 € adulte étranger, ≈ 7 € résident béninois (anciens tarifs), + véhicule et guide</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>eleve</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>faune, nature, aventure</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4708,6 +6932,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>culture, histoire</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4750,6 +6999,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>demi_journee</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>nature, aventure, detente</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4797,6 +7071,31 @@
           <t>+229 97 54 06 56</t>
         </is>
       </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>solo, famille</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4850,6 +7149,31 @@
       <c r="M44" t="n">
         <v>5</v>
       </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>solo</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4897,6 +7221,31 @@
           <t>+229 66 03 37 51</t>
         </is>
       </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>solo</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4939,6 +7288,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>journee</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>nature, faune, aventure</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>amis</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4981,6 +7355,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>solo, couple</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -5029,6 +7428,31 @@
       <c r="M48" t="n">
         <v>6</v>
       </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>solo, couple, famille</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -5077,6 +7501,31 @@
       <c r="M49" t="n">
         <v>5</v>
       </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>detente, culture</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>solo, couple</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -5134,6 +7583,31 @@
           <t>https://tourisme.parakou.bj/2024/01/18/musee-plein-air-et-ethnographique/</t>
         </is>
       </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>courte</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>culture, art</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>solo, couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -5176,6 +7650,31 @@
           <t>Vérifié (Google Places)</t>
         </is>
       </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>economique</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>detente</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>solo</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -5223,6 +7722,36 @@
           <t>Créneaux recommandés 6h-11h et 16h-tombée de la nuit</t>
         </is>
       </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Entrée ≈ 10 000 FCFA / 24 h, + véhicule (≈ 60 000 à 70 000 FCFA), guide (≈ 20 000 FCFA) et carburant</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>eleve</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>sejour</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>faune, nature, aventure</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>couple, amis, famille</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="G53" t="inlineStr">
@@ -5233,6 +7762,20 @@
     </row>
     <row r="54">
       <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=12.0408333,3.0341667</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=11.8523034,3.389122</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="G56" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=12.0408333,3.0341667</t>
         </is>

</xml_diff>

<commit_message>
Créer sa sortie : pause repas dans les lieux avec restauration, catégories vides masquées
OpenStreetMap reste injoignable depuis le cloud (overpass-api.de coupe les
connexions, miroirs sans réponse) : la pause repas utilise en attendant les
8 lieux dont la description sourcée mentionne un restaurant sur place
(hôtels-restaurants, Centre Songhaï), nouvelle colonne « Restauration sur
place » / champ `restauration`. Le prix connu d'un hôtel étant celui de la
nuit, il n'est ni filtré ni compté pour un repas.

Pas de pause repas hors 11h-14h30 (activité à la journée qui inclut le
repas). Catégorie « Restaurants » encore vide : masquée des filtres et du
sitemap, page en 404 tant qu'elle n'a pas de lieu. Générateur SQL en
upsert (insère les lieux nouveaux), testé deux fois sur un Postgres local
dans l'état de la base de prod : id inchangés.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRtuV2T5j4ZnKKUy5a7yX4
</commit_message>
<xml_diff>
--- a/benin_contenu_curation.xlsx
+++ b/benin_contenu_curation.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y43"/>
+  <dimension ref="A1:Z43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -629,6 +629,11 @@
           <t>Photo source</t>
         </is>
       </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Restauration sur place</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1932,6 +1937,11 @@
         </is>
       </c>
       <c r="U15" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -4099,7 +4109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X56"/>
+  <dimension ref="A1:Y56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4233,6 +4243,11 @@
           <t>Photo source</t>
         </is>
       </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Restauration sur place</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -5268,6 +5283,11 @@
           <t>non</t>
         </is>
       </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5561,6 +5581,11 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6216,6 +6241,11 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -6371,6 +6401,11 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -6685,6 +6720,11 @@
           <t>https://commons.wikimedia.org/wiki/File:Grand-Popo-Awal%C3%A9_Plage.jpg</t>
         </is>
       </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -7057,6 +7097,11 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -7537,6 +7582,11 @@
         </is>
       </c>
       <c r="T43" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="Y43" t="inlineStr">
         <is>
           <t>oui</t>
         </is>

</xml_diff>